<commit_message>
Removed Cero-Rehab-Ratios and improved to 96.9
</commit_message>
<xml_diff>
--- a/lmc_estimator_ml/Comps Database.xlsx
+++ b/lmc_estimator_ml/Comps Database.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sergio LMC\EstimatorProjectWebsite\lmc_estimator_ml\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4AA18B4-8491-4B59-8C74-0683502E455D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09CCB71E-7F38-4A68-B09E-1098F5B4A69C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22260,7 +22260,10 @@
         <v>0</v>
       </c>
       <c r="L176">
-        <v>64</v>
+        <v>3</v>
+      </c>
+      <c r="M176">
+        <v>2</v>
       </c>
       <c r="O176" t="s">
         <v>33</v>
@@ -24663,7 +24666,7 @@
         <v>0</v>
       </c>
       <c r="L206">
-        <v>64</v>
+        <v>0</v>
       </c>
       <c r="M206">
         <v>0</v>
@@ -33259,7 +33262,10 @@
         <v>0</v>
       </c>
       <c r="L313">
-        <v>64</v>
+        <v>4</v>
+      </c>
+      <c r="M313">
+        <v>3</v>
       </c>
       <c r="N313">
         <v>843</v>
@@ -59534,6 +59540,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003A09B6389F205A42A2A973C1334F9D95" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ddb9274b495c1a29b7fd082d12db2714">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="36a3c6bc-28c8-4ddd-b997-3b089d610125" xmlns:ns3="fe1b0ca9-8a39-4f9d-9011-9496d0c6acf4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e9cd149fd8a9443b9c8b5edb2d9be73c" ns2:_="" ns3:_="">
     <xsd:import namespace="36a3c6bc-28c8-4ddd-b997-3b089d610125"/>
@@ -59768,15 +59783,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -59789,6 +59795,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{66D2E251-427D-44B3-BDDF-848007EF0934}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8F3E24C7-5934-4EAC-945A-205D26E18EE2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -59807,14 +59821,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{66D2E251-427D-44B3-BDDF-848007EF0934}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{936AAB8D-2AF5-4398-8C2C-BC62676C2253}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Square Foot equals cero drop filet added. 97.38, MAE 22K, RMSE 34K
</commit_message>
<xml_diff>
--- a/lmc_estimator_ml/Comps Database.xlsx
+++ b/lmc_estimator_ml/Comps Database.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sergio LMC\EstimatorProjectWebsite\lmc_estimator_ml\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09CCB71E-7F38-4A68-B09E-1098F5B4A69C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25BBC8D3-02F3-4ED7-8867-88BB94D39F84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Full Internal Comps" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Full Internal Comps'!$A$1:$AA$643</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Full Internal Comps'!$A$1:$AA$657</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6382" uniqueCount="2564">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6508" uniqueCount="2610">
   <si>
     <t>Comp/Property</t>
   </si>
@@ -7728,6 +7728,144 @@
   </si>
   <si>
     <t>2025-10-08 14:27:51</t>
+  </si>
+  <si>
+    <t>L20254932</t>
+  </si>
+  <si>
+    <t>1824 Jessica Ct</t>
+  </si>
+  <si>
+    <t>Winter Park</t>
+  </si>
+  <si>
+    <t>2025-11-10 09:07:44</t>
+  </si>
+  <si>
+    <t>L20254967</t>
+  </si>
+  <si>
+    <t>5752 Janet Dr</t>
+  </si>
+  <si>
+    <t>Iron Station</t>
+  </si>
+  <si>
+    <t>2025-11-10 14:37:15</t>
+  </si>
+  <si>
+    <t>L20254988</t>
+  </si>
+  <si>
+    <t>401 McDonald Ave</t>
+  </si>
+  <si>
+    <t>2025-11-13 09:03:58</t>
+  </si>
+  <si>
+    <t>L20254981</t>
+  </si>
+  <si>
+    <t>1443 Academy St</t>
+  </si>
+  <si>
+    <t>2025-11-13 09:55:00</t>
+  </si>
+  <si>
+    <t>L20254979</t>
+  </si>
+  <si>
+    <t>2333 Wensley Dr</t>
+  </si>
+  <si>
+    <t>2025-11-14 08:12:48</t>
+  </si>
+  <si>
+    <t>L20254977</t>
+  </si>
+  <si>
+    <t>1804 Sheffield Ct</t>
+  </si>
+  <si>
+    <t>2025-11-14 09:42:45</t>
+  </si>
+  <si>
+    <t>L20254966</t>
+  </si>
+  <si>
+    <t>1142 Lockbourne Rd</t>
+  </si>
+  <si>
+    <t>2025-11-14 14:11:05</t>
+  </si>
+  <si>
+    <t>L20254993</t>
+  </si>
+  <si>
+    <t>4152 Cedar Knoll Dr</t>
+  </si>
+  <si>
+    <t>Tucker</t>
+  </si>
+  <si>
+    <t>2025-11-14 14:16:56</t>
+  </si>
+  <si>
+    <t>L20254992</t>
+  </si>
+  <si>
+    <t>7310 Drexel Dr</t>
+  </si>
+  <si>
+    <t>2025-11-14 14:33:53</t>
+  </si>
+  <si>
+    <t>L20254982</t>
+  </si>
+  <si>
+    <t>2 Chaumont Sq NW</t>
+  </si>
+  <si>
+    <t>2025-11-14 16:45:59</t>
+  </si>
+  <si>
+    <t>L20254986</t>
+  </si>
+  <si>
+    <t>6053 Timberwood Trl</t>
+  </si>
+  <si>
+    <t>2025-11-17 13:52:51</t>
+  </si>
+  <si>
+    <t>L20254924</t>
+  </si>
+  <si>
+    <t>197 York St</t>
+  </si>
+  <si>
+    <t>Chester</t>
+  </si>
+  <si>
+    <t>2025-11-19 12:19:47</t>
+  </si>
+  <si>
+    <t>L20254990</t>
+  </si>
+  <si>
+    <t>LOT 79 Kingswood Dr</t>
+  </si>
+  <si>
+    <t>2025-11-19 12:47:45</t>
+  </si>
+  <si>
+    <t>L20255000</t>
+  </si>
+  <si>
+    <t>333 S State Ave</t>
+  </si>
+  <si>
+    <t>2025-11-19 15:45:37</t>
   </si>
 </sst>
 </file>
@@ -8091,7 +8229,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AA643"/>
+  <dimension ref="A1:AA657"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
@@ -59533,22 +59671,1049 @@
         <v>180000</v>
       </c>
     </row>
+    <row r="644" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A644" t="s">
+        <v>27</v>
+      </c>
+      <c r="B644" t="s">
+        <v>2564</v>
+      </c>
+      <c r="C644">
+        <v>1187288</v>
+      </c>
+      <c r="D644" t="s">
+        <v>2565</v>
+      </c>
+      <c r="E644" t="s">
+        <v>2566</v>
+      </c>
+      <c r="F644" t="s">
+        <v>147</v>
+      </c>
+      <c r="G644">
+        <v>32789</v>
+      </c>
+      <c r="H644">
+        <v>2582</v>
+      </c>
+      <c r="I644" t="s">
+        <v>32</v>
+      </c>
+      <c r="J644">
+        <v>911400</v>
+      </c>
+      <c r="K644">
+        <v>352.982184353214</v>
+      </c>
+      <c r="L644">
+        <v>3</v>
+      </c>
+      <c r="M644">
+        <v>2</v>
+      </c>
+      <c r="O644" t="s">
+        <v>33</v>
+      </c>
+      <c r="P644">
+        <v>28.579964</v>
+      </c>
+      <c r="Q644">
+        <v>-81.329859999999996</v>
+      </c>
+      <c r="R644">
+        <v>0.34435261707988901</v>
+      </c>
+      <c r="S644" t="s">
+        <v>34</v>
+      </c>
+      <c r="T644">
+        <v>1983</v>
+      </c>
+      <c r="U644">
+        <v>911400</v>
+      </c>
+      <c r="X644" t="s">
+        <v>2567</v>
+      </c>
+      <c r="Y644">
+        <v>1050000</v>
+      </c>
+      <c r="Z644">
+        <v>130000</v>
+      </c>
+      <c r="AA644">
+        <v>700000</v>
+      </c>
+    </row>
+    <row r="645" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A645" t="s">
+        <v>27</v>
+      </c>
+      <c r="B645" t="s">
+        <v>2568</v>
+      </c>
+      <c r="C645">
+        <v>1187938</v>
+      </c>
+      <c r="D645" t="s">
+        <v>2569</v>
+      </c>
+      <c r="E645" t="s">
+        <v>2570</v>
+      </c>
+      <c r="F645" t="s">
+        <v>40</v>
+      </c>
+      <c r="G645">
+        <v>28080</v>
+      </c>
+      <c r="H645">
+        <v>1950</v>
+      </c>
+      <c r="I645" t="s">
+        <v>62</v>
+      </c>
+      <c r="J645">
+        <v>173000</v>
+      </c>
+      <c r="K645">
+        <v>88.717948717948701</v>
+      </c>
+      <c r="L645">
+        <v>3</v>
+      </c>
+      <c r="M645">
+        <v>3</v>
+      </c>
+      <c r="N645">
+        <v>961</v>
+      </c>
+      <c r="O645" t="s">
+        <v>33</v>
+      </c>
+      <c r="P645">
+        <v>35.481822999999999</v>
+      </c>
+      <c r="Q645">
+        <v>-81.099365000000006</v>
+      </c>
+      <c r="R645">
+        <v>0</v>
+      </c>
+      <c r="S645" t="s">
+        <v>47</v>
+      </c>
+      <c r="T645">
+        <v>1989</v>
+      </c>
+      <c r="U645">
+        <v>390300</v>
+      </c>
+      <c r="X645" t="s">
+        <v>2571</v>
+      </c>
+      <c r="Y645">
+        <v>390000</v>
+      </c>
+      <c r="Z645">
+        <v>65000</v>
+      </c>
+      <c r="AA645">
+        <v>173000</v>
+      </c>
+    </row>
+    <row r="646" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A646" t="s">
+        <v>27</v>
+      </c>
+      <c r="B646" t="s">
+        <v>2572</v>
+      </c>
+      <c r="C646">
+        <v>1188659</v>
+      </c>
+      <c r="D646" t="s">
+        <v>2573</v>
+      </c>
+      <c r="E646" t="s">
+        <v>39</v>
+      </c>
+      <c r="F646" t="s">
+        <v>40</v>
+      </c>
+      <c r="G646">
+        <v>28203</v>
+      </c>
+      <c r="H646">
+        <v>1677</v>
+      </c>
+      <c r="I646" t="s">
+        <v>127</v>
+      </c>
+      <c r="J646">
+        <v>975000</v>
+      </c>
+      <c r="K646">
+        <v>581.39534883720899</v>
+      </c>
+      <c r="L646">
+        <v>3</v>
+      </c>
+      <c r="M646">
+        <v>2</v>
+      </c>
+      <c r="N646">
+        <v>5</v>
+      </c>
+      <c r="O646" t="s">
+        <v>33</v>
+      </c>
+      <c r="P646">
+        <v>35.206000000000003</v>
+      </c>
+      <c r="Q646">
+        <v>-80.857506000000001</v>
+      </c>
+      <c r="R646">
+        <v>0.2</v>
+      </c>
+      <c r="S646" t="s">
+        <v>34</v>
+      </c>
+      <c r="T646">
+        <v>1942</v>
+      </c>
+      <c r="U646">
+        <v>951000</v>
+      </c>
+      <c r="X646" t="s">
+        <v>2574</v>
+      </c>
+      <c r="Y646">
+        <v>2600000</v>
+      </c>
+      <c r="Z646">
+        <v>1000000</v>
+      </c>
+      <c r="AA646">
+        <v>975000</v>
+      </c>
+    </row>
+    <row r="647" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A647" t="s">
+        <v>27</v>
+      </c>
+      <c r="B647" t="s">
+        <v>2575</v>
+      </c>
+      <c r="C647">
+        <v>1188381</v>
+      </c>
+      <c r="D647" t="s">
+        <v>2576</v>
+      </c>
+      <c r="E647" t="s">
+        <v>39</v>
+      </c>
+      <c r="F647" t="s">
+        <v>40</v>
+      </c>
+      <c r="G647">
+        <v>28205</v>
+      </c>
+      <c r="H647">
+        <v>1705</v>
+      </c>
+      <c r="I647" t="s">
+        <v>32</v>
+      </c>
+      <c r="J647">
+        <v>374100</v>
+      </c>
+      <c r="K647">
+        <v>219.41348973607001</v>
+      </c>
+      <c r="L647">
+        <v>2</v>
+      </c>
+      <c r="M647">
+        <v>2</v>
+      </c>
+      <c r="O647" t="s">
+        <v>181</v>
+      </c>
+      <c r="P647">
+        <v>35.241633999999998</v>
+      </c>
+      <c r="Q647">
+        <v>-80.791916000000001</v>
+      </c>
+      <c r="R647">
+        <v>5662</v>
+      </c>
+      <c r="S647" t="s">
+        <v>47</v>
+      </c>
+      <c r="T647">
+        <v>1956</v>
+      </c>
+      <c r="U647">
+        <v>374100</v>
+      </c>
+      <c r="X647" t="s">
+        <v>2577</v>
+      </c>
+      <c r="Y647">
+        <v>600000</v>
+      </c>
+      <c r="Z647">
+        <v>120000</v>
+      </c>
+      <c r="AA647">
+        <v>375000</v>
+      </c>
+    </row>
+    <row r="648" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A648" t="s">
+        <v>27</v>
+      </c>
+      <c r="B648" t="s">
+        <v>2578</v>
+      </c>
+      <c r="C648">
+        <v>1188237</v>
+      </c>
+      <c r="D648" t="s">
+        <v>2579</v>
+      </c>
+      <c r="E648" t="s">
+        <v>39</v>
+      </c>
+      <c r="F648" t="s">
+        <v>40</v>
+      </c>
+      <c r="G648">
+        <v>28210</v>
+      </c>
+      <c r="H648">
+        <v>1950</v>
+      </c>
+      <c r="I648" t="s">
+        <v>90</v>
+      </c>
+      <c r="J648">
+        <v>660000</v>
+      </c>
+      <c r="K648">
+        <v>338.461538461538</v>
+      </c>
+      <c r="L648">
+        <v>4</v>
+      </c>
+      <c r="M648">
+        <v>2.5</v>
+      </c>
+      <c r="N648">
+        <v>55</v>
+      </c>
+      <c r="O648" t="s">
+        <v>33</v>
+      </c>
+      <c r="P648">
+        <v>35.152299999999997</v>
+      </c>
+      <c r="Q648">
+        <v>-80.858770000000007</v>
+      </c>
+      <c r="R648">
+        <v>0.67998163452708904</v>
+      </c>
+      <c r="S648" t="s">
+        <v>34</v>
+      </c>
+      <c r="T648">
+        <v>1960</v>
+      </c>
+      <c r="U648">
+        <v>711600</v>
+      </c>
+      <c r="X648" t="s">
+        <v>2580</v>
+      </c>
+      <c r="Y648">
+        <v>720000</v>
+      </c>
+      <c r="Z648">
+        <v>0</v>
+      </c>
+      <c r="AA648">
+        <v>430000</v>
+      </c>
+    </row>
+    <row r="649" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A649" t="s">
+        <v>27</v>
+      </c>
+      <c r="B649" t="s">
+        <v>2581</v>
+      </c>
+      <c r="C649">
+        <v>1188217</v>
+      </c>
+      <c r="D649" t="s">
+        <v>2582</v>
+      </c>
+      <c r="E649" t="s">
+        <v>105</v>
+      </c>
+      <c r="F649" t="s">
+        <v>31</v>
+      </c>
+      <c r="G649">
+        <v>30815</v>
+      </c>
+      <c r="H649">
+        <v>1278</v>
+      </c>
+      <c r="I649" t="s">
+        <v>32</v>
+      </c>
+      <c r="J649">
+        <v>187900</v>
+      </c>
+      <c r="K649">
+        <v>147.02660406885701</v>
+      </c>
+      <c r="L649">
+        <v>3</v>
+      </c>
+      <c r="M649">
+        <v>2</v>
+      </c>
+      <c r="N649">
+        <v>2190</v>
+      </c>
+      <c r="O649" t="s">
+        <v>33</v>
+      </c>
+      <c r="P649">
+        <v>33.325992999999997</v>
+      </c>
+      <c r="Q649">
+        <v>-82.019419999999997</v>
+      </c>
+      <c r="R649">
+        <v>0.40998622589531603</v>
+      </c>
+      <c r="S649" t="s">
+        <v>34</v>
+      </c>
+      <c r="T649">
+        <v>2001</v>
+      </c>
+      <c r="U649">
+        <v>187900</v>
+      </c>
+      <c r="X649" t="s">
+        <v>2583</v>
+      </c>
+      <c r="Y649">
+        <v>200000</v>
+      </c>
+      <c r="Z649">
+        <v>30000</v>
+      </c>
+      <c r="AA649">
+        <v>134000</v>
+      </c>
+    </row>
+    <row r="650" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A650" t="s">
+        <v>27</v>
+      </c>
+      <c r="B650" t="s">
+        <v>2584</v>
+      </c>
+      <c r="C650">
+        <v>1187891</v>
+      </c>
+      <c r="D650" t="s">
+        <v>2585</v>
+      </c>
+      <c r="E650" t="s">
+        <v>157</v>
+      </c>
+      <c r="F650" t="s">
+        <v>158</v>
+      </c>
+      <c r="G650">
+        <v>43206</v>
+      </c>
+      <c r="H650">
+        <v>1306</v>
+      </c>
+      <c r="I650" t="s">
+        <v>32</v>
+      </c>
+      <c r="J650">
+        <v>193900</v>
+      </c>
+      <c r="K650">
+        <v>351.268115942029</v>
+      </c>
+      <c r="L650">
+        <v>4</v>
+      </c>
+      <c r="M650">
+        <v>1</v>
+      </c>
+      <c r="N650">
+        <v>6956</v>
+      </c>
+      <c r="O650" t="s">
+        <v>33</v>
+      </c>
+      <c r="P650">
+        <v>39.942574</v>
+      </c>
+      <c r="Q650">
+        <v>-82.963319999999996</v>
+      </c>
+      <c r="R650">
+        <v>7480</v>
+      </c>
+      <c r="S650" t="s">
+        <v>47</v>
+      </c>
+      <c r="T650">
+        <v>1928</v>
+      </c>
+      <c r="U650">
+        <v>193900</v>
+      </c>
+      <c r="X650" t="s">
+        <v>2586</v>
+      </c>
+      <c r="Y650">
+        <v>235000</v>
+      </c>
+      <c r="Z650">
+        <v>39000</v>
+      </c>
+      <c r="AA650">
+        <v>152000</v>
+      </c>
+    </row>
+    <row r="651" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A651" t="s">
+        <v>27</v>
+      </c>
+      <c r="B651" t="s">
+        <v>2587</v>
+      </c>
+      <c r="C651">
+        <v>1188753</v>
+      </c>
+      <c r="D651" t="s">
+        <v>2588</v>
+      </c>
+      <c r="E651" t="s">
+        <v>2589</v>
+      </c>
+      <c r="F651" t="s">
+        <v>31</v>
+      </c>
+      <c r="G651">
+        <v>30084</v>
+      </c>
+      <c r="H651">
+        <v>1684</v>
+      </c>
+      <c r="I651" t="s">
+        <v>32</v>
+      </c>
+      <c r="J651">
+        <v>320000</v>
+      </c>
+      <c r="K651">
+        <v>190.02375296912101</v>
+      </c>
+      <c r="L651">
+        <v>3</v>
+      </c>
+      <c r="M651">
+        <v>2</v>
+      </c>
+      <c r="O651" t="s">
+        <v>33</v>
+      </c>
+      <c r="P651">
+        <v>33.831417000000002</v>
+      </c>
+      <c r="Q651">
+        <v>-84.219440000000006</v>
+      </c>
+      <c r="R651">
+        <v>0.45998622589531601</v>
+      </c>
+      <c r="S651" t="s">
+        <v>34</v>
+      </c>
+      <c r="T651">
+        <v>1964</v>
+      </c>
+      <c r="U651">
+        <v>320000</v>
+      </c>
+      <c r="X651" t="s">
+        <v>2590</v>
+      </c>
+      <c r="Y651">
+        <v>480000</v>
+      </c>
+      <c r="Z651">
+        <v>90000</v>
+      </c>
+      <c r="AA651">
+        <v>310000</v>
+      </c>
+    </row>
+    <row r="652" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A652" t="s">
+        <v>27</v>
+      </c>
+      <c r="B652" t="s">
+        <v>2591</v>
+      </c>
+      <c r="C652">
+        <v>1188748</v>
+      </c>
+      <c r="D652" t="s">
+        <v>2592</v>
+      </c>
+      <c r="E652" t="s">
+        <v>45</v>
+      </c>
+      <c r="F652" t="s">
+        <v>46</v>
+      </c>
+      <c r="G652">
+        <v>63130</v>
+      </c>
+      <c r="H652">
+        <v>1871</v>
+      </c>
+      <c r="I652" t="s">
+        <v>32</v>
+      </c>
+      <c r="J652">
+        <v>322600</v>
+      </c>
+      <c r="K652">
+        <v>172.42116515232399</v>
+      </c>
+      <c r="L652">
+        <v>3</v>
+      </c>
+      <c r="M652">
+        <v>1.5</v>
+      </c>
+      <c r="O652" t="s">
+        <v>33</v>
+      </c>
+      <c r="P652">
+        <v>38.666992</v>
+      </c>
+      <c r="Q652">
+        <v>-90.325209999999998</v>
+      </c>
+      <c r="R652">
+        <v>5793</v>
+      </c>
+      <c r="S652" t="s">
+        <v>47</v>
+      </c>
+      <c r="T652">
+        <v>1933</v>
+      </c>
+      <c r="U652">
+        <v>322600</v>
+      </c>
+      <c r="X652" t="s">
+        <v>2593</v>
+      </c>
+      <c r="Y652">
+        <v>435000</v>
+      </c>
+      <c r="Z652">
+        <v>0</v>
+      </c>
+      <c r="AA652">
+        <v>235000</v>
+      </c>
+    </row>
+    <row r="653" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A653" t="s">
+        <v>27</v>
+      </c>
+      <c r="B653" t="s">
+        <v>2594</v>
+      </c>
+      <c r="C653">
+        <v>1188388</v>
+      </c>
+      <c r="D653" t="s">
+        <v>2595</v>
+      </c>
+      <c r="E653" t="s">
+        <v>72</v>
+      </c>
+      <c r="F653" t="s">
+        <v>31</v>
+      </c>
+      <c r="G653">
+        <v>30327</v>
+      </c>
+      <c r="H653">
+        <v>1288</v>
+      </c>
+      <c r="I653" t="s">
+        <v>32</v>
+      </c>
+      <c r="J653">
+        <v>249300</v>
+      </c>
+      <c r="K653">
+        <v>193.55590062111801</v>
+      </c>
+      <c r="L653">
+        <v>2</v>
+      </c>
+      <c r="M653">
+        <v>2.5</v>
+      </c>
+      <c r="N653">
+        <v>10800</v>
+      </c>
+      <c r="O653" t="s">
+        <v>969</v>
+      </c>
+      <c r="P653">
+        <v>33.823444000000002</v>
+      </c>
+      <c r="Q653">
+        <v>-84.424164000000005</v>
+      </c>
+      <c r="R653">
+        <v>1289</v>
+      </c>
+      <c r="S653" t="s">
+        <v>47</v>
+      </c>
+      <c r="T653">
+        <v>1968</v>
+      </c>
+      <c r="U653">
+        <v>249300</v>
+      </c>
+      <c r="X653" t="s">
+        <v>2596</v>
+      </c>
+      <c r="Y653">
+        <v>285000</v>
+      </c>
+      <c r="Z653">
+        <v>25000</v>
+      </c>
+      <c r="AA653">
+        <v>206500</v>
+      </c>
+    </row>
+    <row r="654" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A654" t="s">
+        <v>27</v>
+      </c>
+      <c r="B654" t="s">
+        <v>2597</v>
+      </c>
+      <c r="C654">
+        <v>1188638</v>
+      </c>
+      <c r="D654" t="s">
+        <v>2598</v>
+      </c>
+      <c r="E654" t="s">
+        <v>1684</v>
+      </c>
+      <c r="F654" t="s">
+        <v>40</v>
+      </c>
+      <c r="G654">
+        <v>27284</v>
+      </c>
+      <c r="H654">
+        <v>1508</v>
+      </c>
+      <c r="I654" t="s">
+        <v>32</v>
+      </c>
+      <c r="J654">
+        <v>223900</v>
+      </c>
+      <c r="K654">
+        <v>148.47480106100701</v>
+      </c>
+      <c r="L654">
+        <v>3</v>
+      </c>
+      <c r="M654">
+        <v>2</v>
+      </c>
+      <c r="N654">
+        <v>4026</v>
+      </c>
+      <c r="O654" t="s">
+        <v>33</v>
+      </c>
+      <c r="P654">
+        <v>36.126728</v>
+      </c>
+      <c r="Q654">
+        <v>-80.103324999999998</v>
+      </c>
+      <c r="R654">
+        <v>0.72998163452708897</v>
+      </c>
+      <c r="S654" t="s">
+        <v>34</v>
+      </c>
+      <c r="T654">
+        <v>1979</v>
+      </c>
+      <c r="U654">
+        <v>223900</v>
+      </c>
+      <c r="X654" t="s">
+        <v>2599</v>
+      </c>
+      <c r="Y654">
+        <v>290000</v>
+      </c>
+      <c r="Z654">
+        <v>60000</v>
+      </c>
+      <c r="AA654">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="655" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A655" t="s">
+        <v>27</v>
+      </c>
+      <c r="B655" t="s">
+        <v>2600</v>
+      </c>
+      <c r="C655">
+        <v>1187120</v>
+      </c>
+      <c r="D655" t="s">
+        <v>2601</v>
+      </c>
+      <c r="E655" t="s">
+        <v>2602</v>
+      </c>
+      <c r="F655" t="s">
+        <v>84</v>
+      </c>
+      <c r="G655">
+        <v>29706</v>
+      </c>
+      <c r="I655" t="s">
+        <v>90</v>
+      </c>
+      <c r="J655">
+        <v>7000</v>
+      </c>
+      <c r="K655">
+        <v>0</v>
+      </c>
+      <c r="N655">
+        <v>325</v>
+      </c>
+      <c r="O655" t="s">
+        <v>91</v>
+      </c>
+      <c r="P655">
+        <v>34.716952999999997</v>
+      </c>
+      <c r="Q655">
+        <v>-81.205820000000003</v>
+      </c>
+      <c r="R655">
+        <v>0.13</v>
+      </c>
+      <c r="S655" t="s">
+        <v>34</v>
+      </c>
+      <c r="X655" t="s">
+        <v>2603</v>
+      </c>
+      <c r="Y655">
+        <v>180000</v>
+      </c>
+      <c r="Z655">
+        <v>125000</v>
+      </c>
+      <c r="AA655">
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="656" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A656" t="s">
+        <v>27</v>
+      </c>
+      <c r="B656" t="s">
+        <v>2604</v>
+      </c>
+      <c r="C656">
+        <v>1188703</v>
+      </c>
+      <c r="D656" t="s">
+        <v>2605</v>
+      </c>
+      <c r="E656" t="s">
+        <v>67</v>
+      </c>
+      <c r="F656" t="s">
+        <v>40</v>
+      </c>
+      <c r="G656">
+        <v>28625</v>
+      </c>
+      <c r="I656" t="s">
+        <v>127</v>
+      </c>
+      <c r="J656">
+        <v>25000</v>
+      </c>
+      <c r="K656">
+        <v>0</v>
+      </c>
+      <c r="N656">
+        <v>3</v>
+      </c>
+      <c r="O656" t="s">
+        <v>91</v>
+      </c>
+      <c r="P656">
+        <v>35.844119999999997</v>
+      </c>
+      <c r="Q656">
+        <v>-80.881584000000004</v>
+      </c>
+      <c r="R656">
+        <v>0.46</v>
+      </c>
+      <c r="S656" t="s">
+        <v>34</v>
+      </c>
+      <c r="X656" t="s">
+        <v>2606</v>
+      </c>
+      <c r="Y656">
+        <v>380000</v>
+      </c>
+      <c r="Z656">
+        <v>192050</v>
+      </c>
+      <c r="AA656">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="657" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A657" t="s">
+        <v>27</v>
+      </c>
+      <c r="B657" t="s">
+        <v>2607</v>
+      </c>
+      <c r="C657">
+        <v>1189079</v>
+      </c>
+      <c r="D657" t="s">
+        <v>2608</v>
+      </c>
+      <c r="E657" t="s">
+        <v>163</v>
+      </c>
+      <c r="F657" t="s">
+        <v>164</v>
+      </c>
+      <c r="G657">
+        <v>46201</v>
+      </c>
+      <c r="H657">
+        <v>1200</v>
+      </c>
+      <c r="I657" t="s">
+        <v>90</v>
+      </c>
+      <c r="J657">
+        <v>100000</v>
+      </c>
+      <c r="K657">
+        <v>83.3333333333333</v>
+      </c>
+      <c r="L657">
+        <v>2</v>
+      </c>
+      <c r="M657">
+        <v>2</v>
+      </c>
+      <c r="N657">
+        <v>356</v>
+      </c>
+      <c r="O657" t="s">
+        <v>181</v>
+      </c>
+      <c r="P657">
+        <v>39.761189999999999</v>
+      </c>
+      <c r="Q657">
+        <v>-86.130240000000001</v>
+      </c>
+      <c r="R657">
+        <v>4443</v>
+      </c>
+      <c r="S657" t="s">
+        <v>47</v>
+      </c>
+      <c r="T657">
+        <v>1910</v>
+      </c>
+      <c r="U657">
+        <v>100900</v>
+      </c>
+      <c r="X657" t="s">
+        <v>2609</v>
+      </c>
+      <c r="Y657">
+        <v>275000</v>
+      </c>
+      <c r="Z657">
+        <v>0</v>
+      </c>
+      <c r="AA657">
+        <v>120000</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AA643" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:AA657" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003A09B6389F205A42A2A973C1334F9D95" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ddb9274b495c1a29b7fd082d12db2714">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="36a3c6bc-28c8-4ddd-b997-3b089d610125" xmlns:ns3="fe1b0ca9-8a39-4f9d-9011-9496d0c6acf4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e9cd149fd8a9443b9c8b5edb2d9be73c" ns2:_="" ns3:_="">
     <xsd:import namespace="36a3c6bc-28c8-4ddd-b997-3b089d610125"/>
@@ -59783,6 +60948,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -59795,14 +60969,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{66D2E251-427D-44B3-BDDF-848007EF0934}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8F3E24C7-5934-4EAC-945A-205D26E18EE2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -59821,6 +60987,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{66D2E251-427D-44B3-BDDF-848007EF0934}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{936AAB8D-2AF5-4398-8C2C-BC62676C2253}">
   <ds:schemaRefs>

</xml_diff>